<commit_message>
Review correction: fire extinguishers are on all 47 buildings as accessory quantities; building labour at card $29,730.96
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GNRrrx1C9yJ5N627f7yfrr
</commit_message>
<xml_diff>
--- a/03_GC500_Delivery_Control/review_22Oct2026_baseplan6_schedule13/GC500_Baseplan_vs_Record_22Oct2026.xlsx
+++ b/03_GC500_Delivery_Control/review_22Oct2026_baseplan6_schedule13/GC500_Baseplan_vs_Record_22Oct2026.xlsx
@@ -514,12 +514,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>47 buildings ticked on the record: install 47, levelling 47, cleaning 47, demob 47, steps 40 (none on P06, P38, P39, P42, P60, P62, P63), fire extinguisher 10. At the card that is $27,805.11</t>
+          <t>47 buildings ticked on the record: install 47, levelling 47, cleaning 47, demob 47, steps 40 (none on P06, P38, P39, P42, P60, P62, P63), fire extinguisher 47 (one in every building, recorded 20 Oct). At the card that is $29,730.96</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Charge each line by the building, not a flat package: steps only where fitted, fire extinguisher only where supplied. Difference $1,707.24 over on Baseplan as it stands (and it is on 45 buildings where the record has 47)</t>
+          <t>Charge each line by the building, not a flat package: steps only where fitted (40, not 45), and on all 47 buildings, not 45. Net Baseplan is $218.61 under as it stands; demob is in the package before it is done</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -3648,14 +3648,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P2" s="4" t="inlineStr"/>
+      <c r="P2" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q2" s="4" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R2" s="4" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S2" s="4" t="n">
         <v>2</v>
@@ -3742,14 +3746,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P3" s="5" t="inlineStr"/>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q3" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R3" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S3" s="5" t="n">
         <v>2</v>
@@ -3828,14 +3836,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S4" s="2" t="n">
         <v>2</v>
@@ -3922,14 +3934,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P5" s="5" t="inlineStr"/>
+      <c r="P5" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q5" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R5" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S5" s="5" t="n">
         <v>2</v>
@@ -4012,14 +4028,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P6" s="5" t="inlineStr"/>
+      <c r="P6" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q6" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R6" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S6" s="5" t="n">
         <v>2</v>
@@ -4102,14 +4122,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P7" s="5" t="inlineStr"/>
+      <c r="P7" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q7" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R7" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S7" s="5" t="n">
         <v>2</v>
@@ -4192,14 +4216,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P8" s="5" t="inlineStr"/>
+      <c r="P8" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q8" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R8" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S8" s="5" t="n">
         <v>2</v>
@@ -4278,14 +4306,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P9" s="2" t="inlineStr"/>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R9" s="2" t="n">
-        <v>447.63</v>
+        <v>499.68</v>
       </c>
       <c r="S9" s="2" t="n">
         <v>2</v>
@@ -4466,14 +4498,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P11" s="5" t="inlineStr"/>
+      <c r="P11" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q11" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R11" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S11" s="5" t="n">
         <v>2</v>
@@ -4552,14 +4588,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P12" s="5" t="inlineStr"/>
+      <c r="P12" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q12" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R12" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S12" s="5" t="n">
         <v>2</v>
@@ -4638,14 +4678,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P13" s="5" t="inlineStr"/>
+      <c r="P13" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q13" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R13" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S13" s="5" t="n">
         <v>2</v>
@@ -4728,14 +4772,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P14" s="5" t="inlineStr"/>
+      <c r="P14" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q14" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R14" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S14" s="5" t="n">
         <v>2</v>
@@ -4814,14 +4862,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P15" s="5" t="inlineStr"/>
+      <c r="P15" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q15" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R15" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S15" s="5" t="n">
         <v>2</v>
@@ -4900,14 +4952,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P16" s="5" t="inlineStr"/>
+      <c r="P16" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q16" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R16" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S16" s="5" t="n">
         <v>2</v>
@@ -4990,14 +5046,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P17" s="5" t="inlineStr"/>
+      <c r="P17" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q17" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R17" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S17" s="5" t="n">
         <v>2</v>
@@ -5080,14 +5140,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P18" s="5" t="inlineStr"/>
+      <c r="P18" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q18" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R18" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S18" s="5" t="n">
         <v>2</v>
@@ -5170,14 +5234,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P19" s="5" t="inlineStr"/>
+      <c r="P19" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q19" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R19" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S19" s="5" t="n">
         <v>2</v>
@@ -5260,14 +5328,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P20" s="5" t="inlineStr"/>
+      <c r="P20" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q20" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R20" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S20" s="5" t="n">
         <v>2</v>
@@ -5350,14 +5422,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P21" s="5" t="inlineStr"/>
+      <c r="P21" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q21" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R21" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S21" s="5" t="n">
         <v>2</v>
@@ -5440,14 +5516,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P22" s="5" t="inlineStr"/>
+      <c r="P22" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q22" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R22" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S22" s="5" t="n">
         <v>2</v>
@@ -5530,14 +5610,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P23" s="5" t="inlineStr"/>
+      <c r="P23" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q23" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R23" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S23" s="5" t="n">
         <v>2</v>
@@ -5714,14 +5798,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P25" s="5" t="inlineStr"/>
+      <c r="P25" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q25" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R25" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S25" s="5" t="n">
         <v>2</v>
@@ -5800,14 +5888,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P26" s="2" t="inlineStr"/>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q26" s="2" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S26" s="2" t="n">
         <v>2</v>
@@ -5890,14 +5982,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P27" s="5" t="inlineStr"/>
+      <c r="P27" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q27" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R27" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S27" s="5" t="n">
         <v>2</v>
@@ -5976,14 +6072,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P28" s="5" t="inlineStr"/>
+      <c r="P28" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q28" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R28" s="5" t="n">
-        <v>447.63</v>
+        <v>499.68</v>
       </c>
       <c r="S28" s="5" t="n">
         <v>2</v>
@@ -6062,14 +6162,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P29" s="5" t="inlineStr"/>
+      <c r="P29" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q29" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R29" s="5" t="n">
-        <v>447.63</v>
+        <v>499.68</v>
       </c>
       <c r="S29" s="5" t="n">
         <v>2</v>
@@ -6152,14 +6256,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P30" s="5" t="inlineStr"/>
+      <c r="P30" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q30" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R30" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S30" s="5" t="n">
         <v>2</v>
@@ -6238,14 +6346,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P31" s="5" t="inlineStr"/>
+      <c r="P31" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q31" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R31" s="5" t="n">
-        <v>447.63</v>
+        <v>499.68</v>
       </c>
       <c r="S31" s="5" t="n">
         <v>2</v>
@@ -6328,14 +6440,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P32" s="5" t="inlineStr"/>
+      <c r="P32" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q32" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R32" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S32" s="5" t="n">
         <v>2</v>
@@ -6888,14 +7004,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P38" s="5" t="inlineStr"/>
+      <c r="P38" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q38" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R38" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S38" s="5" t="n">
         <v>2</v>
@@ -6978,14 +7098,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P39" s="5" t="inlineStr"/>
+      <c r="P39" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q39" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R39" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S39" s="5" t="n">
         <v>2</v>
@@ -7162,14 +7286,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P41" s="2" t="inlineStr"/>
+      <c r="P41" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q41" s="2" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R41" s="2" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S41" s="2" t="n">
         <v>2</v>
@@ -7252,14 +7380,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P42" s="5" t="inlineStr"/>
+      <c r="P42" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q42" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R42" s="5" t="n">
-        <v>447.63</v>
+        <v>499.68</v>
       </c>
       <c r="S42" s="5" t="n">
         <v>2</v>
@@ -7338,14 +7470,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P43" s="5" t="inlineStr"/>
+      <c r="P43" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q43" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R43" s="5" t="n">
-        <v>447.63</v>
+        <v>499.68</v>
       </c>
       <c r="S43" s="5" t="n">
         <v>2</v>
@@ -7424,14 +7560,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P44" s="5" t="inlineStr"/>
+      <c r="P44" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q44" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R44" s="5" t="n">
-        <v>447.63</v>
+        <v>499.68</v>
       </c>
       <c r="S44" s="5" t="n">
         <v>2</v>
@@ -7514,14 +7654,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P45" s="5" t="inlineStr"/>
+      <c r="P45" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q45" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R45" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S45" s="5" t="n">
         <v>2</v>
@@ -7698,14 +7842,18 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="P47" s="5" t="inlineStr"/>
+      <c r="P47" s="5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="Q47" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
       <c r="R47" s="5" t="n">
-        <v>603.78</v>
+        <v>655.83</v>
       </c>
       <c r="S47" s="5" t="n">
         <v>2</v>

</xml_diff>